<commit_message>
Auto update: 2026-08-30 11:35:52
</commit_message>
<xml_diff>
--- a/docs/成績計算.xlsx
+++ b/docs/成績計算.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Dev\CDY_YAKYULIFE\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3C1FBF72-5330-44B7-9A19-969288F536DA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{91818B18-5C85-4D44-9B22-1AC7440DB131}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3940" yWindow="930" windowWidth="30650" windowHeight="17100" xr2:uid="{AA24EB7E-E109-46F7-B027-D52B85957C16}"/>
+    <workbookView xWindow="2280" yWindow="2280" windowWidth="28800" windowHeight="15910" xr2:uid="{AA24EB7E-E109-46F7-B027-D52B85957C16}"/>
   </bookViews>
   <sheets>
     <sheet name="工作表1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="45">
   <si>
     <t>G</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -138,6 +138,86 @@
   </si>
   <si>
     <t>CS = round(SB * (0.38 - 0.20 * min(1.0, (spd - (par - 59)) / 75.0)) * noise) + round[-1, +1]</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>打者</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>投手</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>G</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>原算式+ round [-3,+3]</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>GS</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>原算式+ round [-2,+2]</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>W</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>L</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>SV</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>HLD</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>IP</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>H</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>R</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>ER</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>BB</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>SO</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>SV = max(0, min(G - GS - W - L, round(65 * ((G - GS) / 65.0) * min(1.05, ((投手評價) - (par - 59)) / 75.0) * noise * (球隊勝率 / 0.500)) + round[-3, +3]))</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>HLD = max(0, min(G - GS - W - L - SV, round(40 * ((G - GS) / 65.0) * min(1.05, ((投手評價) - (par - 59)) / 75.0) * noise * (球隊勝率 / 0.500)) + round[-3, +3]))</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>W = max(0, min(G, round((25 * (GS / 35.0) + 8 * ((G - GS) / 65.0)) * min(1.05, ((投手評價) - (par - 59)) / 75.0) * noise * (球隊勝率 / 0.500)) + round[-2, +2]))</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>L = max(0, min(G - W, round((20 * (GS / 35.0) + 8 * ((G - GS) / 65.0)) * max(0.20, 1.20 - min(1.05, ((投手評價) - (par - 59)) / 75.0)) * noise * ((1.0 - 球隊勝率) / 0.500)) + round[-2, +2]))</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -533,13 +613,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B28A609D-0D8F-490C-9C0F-19DAF045CAC2}">
-  <dimension ref="C2:L15"/>
+  <dimension ref="B2:L29"/>
   <sheetFormatPr defaultRowHeight="17" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="7" max="7" width="157.1796875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="172.1796875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="3:12" x14ac:dyDescent="0.4">
+    <row r="2" spans="2:12" x14ac:dyDescent="0.4">
+      <c r="B2" t="s">
+        <v>25</v>
+      </c>
       <c r="C2" t="s">
         <v>0</v>
       </c>
@@ -547,7 +630,7 @@
         <v>162</v>
       </c>
     </row>
-    <row r="3" spans="3:12" x14ac:dyDescent="0.4">
+    <row r="3" spans="2:12" x14ac:dyDescent="0.4">
       <c r="C3" t="s">
         <v>1</v>
       </c>
@@ -561,7 +644,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="4" spans="3:12" x14ac:dyDescent="0.4">
+    <row r="4" spans="2:12" x14ac:dyDescent="0.4">
       <c r="C4" t="s">
         <v>2</v>
       </c>
@@ -575,7 +658,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="5" spans="3:12" x14ac:dyDescent="0.4">
+    <row r="5" spans="2:12" x14ac:dyDescent="0.4">
       <c r="C5" t="s">
         <v>3</v>
       </c>
@@ -589,7 +672,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="6" spans="3:12" x14ac:dyDescent="0.4">
+    <row r="6" spans="2:12" x14ac:dyDescent="0.4">
       <c r="C6" t="s">
         <v>13</v>
       </c>
@@ -603,7 +686,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="7" spans="3:12" x14ac:dyDescent="0.4">
+    <row r="7" spans="2:12" x14ac:dyDescent="0.4">
       <c r="C7" t="s">
         <v>4</v>
       </c>
@@ -618,7 +701,7 @@
       </c>
       <c r="L7" s="1"/>
     </row>
-    <row r="8" spans="3:12" x14ac:dyDescent="0.4">
+    <row r="8" spans="2:12" x14ac:dyDescent="0.4">
       <c r="C8" t="s">
         <v>5</v>
       </c>
@@ -632,7 +715,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="9" spans="3:12" x14ac:dyDescent="0.4">
+    <row r="9" spans="2:12" x14ac:dyDescent="0.4">
       <c r="C9" t="s">
         <v>6</v>
       </c>
@@ -646,7 +729,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="10" spans="3:12" x14ac:dyDescent="0.4">
+    <row r="10" spans="2:12" x14ac:dyDescent="0.4">
       <c r="C10" t="s">
         <v>7</v>
       </c>
@@ -660,7 +743,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="11" spans="3:12" x14ac:dyDescent="0.4">
+    <row r="11" spans="2:12" x14ac:dyDescent="0.4">
       <c r="C11" t="s">
         <v>8</v>
       </c>
@@ -674,7 +757,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="12" spans="3:12" x14ac:dyDescent="0.4">
+    <row r="12" spans="2:12" x14ac:dyDescent="0.4">
       <c r="C12" t="s">
         <v>9</v>
       </c>
@@ -685,7 +768,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="13" spans="3:12" x14ac:dyDescent="0.4">
+    <row r="13" spans="2:12" x14ac:dyDescent="0.4">
       <c r="C13" t="s">
         <v>10</v>
       </c>
@@ -699,7 +782,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="14" spans="3:12" x14ac:dyDescent="0.4">
+    <row r="14" spans="2:12" x14ac:dyDescent="0.4">
       <c r="C14" t="s">
         <v>11</v>
       </c>
@@ -713,7 +796,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="15" spans="3:12" x14ac:dyDescent="0.4">
+    <row r="15" spans="2:12" x14ac:dyDescent="0.4">
       <c r="C15" t="s">
         <v>12</v>
       </c>
@@ -725,6 +808,117 @@
       </c>
       <c r="G15" t="s">
         <v>24</v>
+      </c>
+    </row>
+    <row r="18" spans="2:7" x14ac:dyDescent="0.4">
+      <c r="B18" t="s">
+        <v>26</v>
+      </c>
+      <c r="C18" t="s">
+        <v>27</v>
+      </c>
+      <c r="G18" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="19" spans="2:7" x14ac:dyDescent="0.4">
+      <c r="C19" t="s">
+        <v>29</v>
+      </c>
+      <c r="G19" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="20" spans="2:7" x14ac:dyDescent="0.4">
+      <c r="C20" t="s">
+        <v>31</v>
+      </c>
+      <c r="E20">
+        <v>25</v>
+      </c>
+      <c r="G20" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="21" spans="2:7" x14ac:dyDescent="0.4">
+      <c r="C21" t="s">
+        <v>32</v>
+      </c>
+      <c r="E21">
+        <v>20</v>
+      </c>
+      <c r="G21" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="22" spans="2:7" x14ac:dyDescent="0.4">
+      <c r="C22" t="s">
+        <v>33</v>
+      </c>
+      <c r="E22">
+        <v>65</v>
+      </c>
+      <c r="G22" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="23" spans="2:7" x14ac:dyDescent="0.4">
+      <c r="C23" t="s">
+        <v>34</v>
+      </c>
+      <c r="E23">
+        <v>40</v>
+      </c>
+      <c r="G23" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="24" spans="2:7" x14ac:dyDescent="0.4">
+      <c r="C24" t="s">
+        <v>35</v>
+      </c>
+      <c r="E24">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="25" spans="2:7" x14ac:dyDescent="0.4">
+      <c r="C25" t="s">
+        <v>36</v>
+      </c>
+      <c r="E25">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="26" spans="2:7" x14ac:dyDescent="0.4">
+      <c r="C26" t="s">
+        <v>37</v>
+      </c>
+      <c r="E26">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="27" spans="2:7" x14ac:dyDescent="0.4">
+      <c r="C27" t="s">
+        <v>38</v>
+      </c>
+      <c r="E27">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="28" spans="2:7" x14ac:dyDescent="0.4">
+      <c r="C28" t="s">
+        <v>39</v>
+      </c>
+      <c r="E28">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="29" spans="2:7" x14ac:dyDescent="0.4">
+      <c r="C29" t="s">
+        <v>40</v>
+      </c>
+      <c r="E29">
+        <v>360</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto update: 2026-09-03 14:32:30
</commit_message>
<xml_diff>
--- a/docs/成績計算.xlsx
+++ b/docs/成績計算.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Dev\CDY_YAKYULIFE\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{91818B18-5C85-4D44-9B22-1AC7440DB131}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4F4A22E6-5399-4B53-A284-0B7080BC2447}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2280" yWindow="2280" windowWidth="28800" windowHeight="15910" xr2:uid="{AA24EB7E-E109-46F7-B027-D52B85957C16}"/>
+    <workbookView xWindow="4160" yWindow="380" windowWidth="28800" windowHeight="15910" xr2:uid="{AA24EB7E-E109-46F7-B027-D52B85957C16}"/>
   </bookViews>
   <sheets>
     <sheet name="工作表1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="45">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="68" uniqueCount="66">
   <si>
     <t>G</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -133,14 +133,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>SO = min(AB, round(220 * (AB / 600.0) * min(1.05, max(0.05, ((pow * 1.2 - con * 1.0 - eye * 0.5) + 112.5 - 0.3 * (par - 59)) / 150.0)) * noise)) + round[-3, +3]</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>CS = round(SB * (0.38 - 0.20 * min(1.0, (spd - (par - 59)) / 75.0)) * noise) + round[-1, +1]</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>打者</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -218,6 +210,98 @@
   </si>
   <si>
     <t>L = max(0, min(G - W, round((20 * (GS / 35.0) + 8 * ((G - GS) / 65.0)) * max(0.20, 1.20 - min(1.05, ((投手評價) - (par - 59)) / 75.0)) * noise * ((1.0 - 球隊勝率) / 0.500)) + round[-2, +2]))</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>考慮信任度</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>IP_SP = max(0, min(GS * 9 + (G - GS) * 3, round((260 * (GS / 35.0) + 70 * ((G - GS) / 65.0)) * min(1.05, max(0.20, (std - (par - 59)) / 75.0)) * noise) + round[-3, +3]))</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>IP_CP = max(0, min(G * 2, round(65 * (G / 65.0) * min(1.05, max(0.85, (std - (par - 59)) / 75.0)) * noise) + round[-3, +3]))</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>IP_SU = max(0, min(G * 2, round(65 * (G / 65.0) * min(1.05, max(0.85, (std - (par - 59)) / 75.0)) * noise) + round[-3, +3]))</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>IP_MR = max(0, min(G * 3, round(55 * (G / 65.0) * min(1.05, max(0.70, (std - (par - 59)) / 75.0)) * noise) + round[-3, +3]))</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>IP_LR = max(0, min(GS * 9 + (G - GS) * 4, round((240 * (GS / 35.0) + 120 * ((G - GS) / 65.0)) * min(1.05, max(0.40, (std - (par - 59)) / 75.0)) * noise) + round[-3, +3]))</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>SO = min(AB - H, round(220 * ((AB - H) / 600.0) * min(1.05, max(0.05, ((pow * 1.2 - con * 1.0 - eye * 0.5) + 112.5 - 0.3 * (par - 59)) / 150.0)) * noise)) + round[-3, +3]</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>現有</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>H = max(0, min(IP * 3, round(260 * (IP / 200.0) * max(0.55, 1.40 - 0.80 * min(1.05, ((投手評價) - (par - 59)) / 75.0)) * noise) + round[-3, +3]))</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>ER = max(0, min(IP * 2, round(140 * (IP / 200.0) * max(0.35, 1.55 - 1.15 * min(1.05, ((投手評價) - (par - 59)) / 75.0)) * noise) + round[-2, +2]))</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>R = ER + max(0, round(12 * (IP / 200.0) * noise) + round[-1, +1])</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>SO = max(0, min(IP * 3, round((50 + 310 * pow(max(0.0, min(1.0, ((1.5 * 球速 + 控球 + 1.5 * 橫向 + 變速) - 5 * (par - 59)) / 375.0)), 3.0)) * (IP / 240.0) * noise) + round[-5, +5]))</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>20-120</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>50-360</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>BB = max(0, min(IP * 2, round((20 + 100 * max(0.0, min(1.0, (75 - (控球 - (par - 59))) / 55.0))) * (IP / 200.0) * noise) + round[-3, +3]))</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>HR</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>HR = max(0, min(H, round((10 + 35 * max(0.0, min(1.0, ((75 - 控球) * 1.5 + (75 - 縱向變) * 1.2 + (75 - 球速) * 0.8 + 橫向變 * 0.4 + 3.1 * (par - 59)) / 220.0))) * (IP / 200.0) * noise) + round[-2, +2]))</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>10-45</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>SB = max(0, min(H + BB + IBB - HR, round(80 * (PA / 720.0) * max(0.0, min(1.0, ((spd - (par - 59)) - 35) / 40.0)) * noise) + round[-3, +3]))</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>CS = round(SB * (0.38 - 0.20 * min(1.0, (spd - (par - 59)) / 75.0)) * noise) + round[-2, +2]</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>投手STD =&gt; 55，SP&gt;LR；STD &lt; 55，CP&gt;SU&gt;MR&gt;LR</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>SP低於PAR 5%時降為LR，CP大於等於PAR*1.05，SU大於等於PAR*1.2，MR大於等於PAR*0.97，LR小於PAR*0.95</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>類似野手的守位降位，養成/二軍也比照野手</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -272,12 +356,15 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -613,7 +700,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B28A609D-0D8F-490C-9C0F-19DAF045CAC2}">
-  <dimension ref="B2:L29"/>
+  <dimension ref="B2:L38"/>
   <sheetFormatPr defaultRowHeight="17" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="7" max="7" width="172.1796875" bestFit="1" customWidth="1"/>
@@ -621,13 +708,16 @@
   <sheetData>
     <row r="2" spans="2:12" x14ac:dyDescent="0.4">
       <c r="B2" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="C2" t="s">
         <v>0</v>
       </c>
       <c r="D2">
         <v>162</v>
+      </c>
+      <c r="H2" t="s">
+        <v>43</v>
       </c>
     </row>
     <row r="3" spans="2:12" x14ac:dyDescent="0.4">
@@ -767,6 +857,9 @@
       <c r="E12">
         <v>120</v>
       </c>
+      <c r="G12" t="s">
+        <v>50</v>
+      </c>
     </row>
     <row r="13" spans="2:12" x14ac:dyDescent="0.4">
       <c r="C13" t="s">
@@ -776,10 +869,10 @@
         <v>223</v>
       </c>
       <c r="E13">
-        <v>240</v>
+        <v>220</v>
       </c>
       <c r="G13" t="s">
-        <v>23</v>
+        <v>49</v>
       </c>
     </row>
     <row r="14" spans="2:12" x14ac:dyDescent="0.4">
@@ -793,7 +886,7 @@
         <v>80</v>
       </c>
       <c r="G14" t="s">
-        <v>16</v>
+        <v>61</v>
       </c>
     </row>
     <row r="15" spans="2:12" x14ac:dyDescent="0.4">
@@ -807,118 +900,188 @@
         <v>30</v>
       </c>
       <c r="G15" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="18" spans="2:8" x14ac:dyDescent="0.4">
+      <c r="B18" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="18" spans="2:7" x14ac:dyDescent="0.4">
-      <c r="B18" t="s">
+      <c r="C18" t="s">
+        <v>25</v>
+      </c>
+      <c r="G18" t="s">
         <v>26</v>
       </c>
-      <c r="C18" t="s">
+      <c r="H18" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="19" spans="2:8" x14ac:dyDescent="0.4">
+      <c r="C19" t="s">
         <v>27</v>
       </c>
-      <c r="G18" t="s">
+      <c r="G19" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="19" spans="2:7" x14ac:dyDescent="0.4">
-      <c r="C19" t="s">
+      <c r="H19" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="20" spans="2:8" x14ac:dyDescent="0.4">
+      <c r="C20" t="s">
         <v>29</v>
-      </c>
-      <c r="G19" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="20" spans="2:7" x14ac:dyDescent="0.4">
-      <c r="C20" t="s">
-        <v>31</v>
       </c>
       <c r="E20">
         <v>25</v>
       </c>
       <c r="G20" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="21" spans="2:7" x14ac:dyDescent="0.4">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="21" spans="2:8" x14ac:dyDescent="0.4">
       <c r="C21" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="E21">
         <v>20</v>
       </c>
       <c r="G21" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="22" spans="2:7" x14ac:dyDescent="0.4">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="22" spans="2:8" x14ac:dyDescent="0.4">
       <c r="C22" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="E22">
         <v>65</v>
       </c>
       <c r="G22" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="23" spans="2:7" x14ac:dyDescent="0.4">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="23" spans="2:8" x14ac:dyDescent="0.4">
       <c r="C23" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="E23">
         <v>40</v>
       </c>
       <c r="G23" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="24" spans="2:7" x14ac:dyDescent="0.4">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="24" spans="2:8" x14ac:dyDescent="0.4">
       <c r="C24" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="E24">
         <v>260</v>
       </c>
-    </row>
-    <row r="25" spans="2:7" x14ac:dyDescent="0.4">
-      <c r="C25" t="s">
+      <c r="G24" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="25" spans="2:8" x14ac:dyDescent="0.4">
+      <c r="G25" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="26" spans="2:8" x14ac:dyDescent="0.4">
+      <c r="G26" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="27" spans="2:8" x14ac:dyDescent="0.4">
+      <c r="G27" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="28" spans="2:8" x14ac:dyDescent="0.4">
+      <c r="G28" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="29" spans="2:8" x14ac:dyDescent="0.4">
+      <c r="C29" t="s">
+        <v>34</v>
+      </c>
+      <c r="E29">
+        <v>260</v>
+      </c>
+      <c r="G29" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="30" spans="2:8" x14ac:dyDescent="0.4">
+      <c r="C30" t="s">
+        <v>35</v>
+      </c>
+      <c r="E30">
+        <v>150</v>
+      </c>
+      <c r="G30" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="31" spans="2:8" x14ac:dyDescent="0.4">
+      <c r="C31" t="s">
         <v>36</v>
       </c>
-      <c r="E25">
-        <v>260</v>
-      </c>
-    </row>
-    <row r="26" spans="2:7" x14ac:dyDescent="0.4">
-      <c r="C26" t="s">
+      <c r="E31">
+        <v>140</v>
+      </c>
+      <c r="G31" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="32" spans="2:8" x14ac:dyDescent="0.4">
+      <c r="C32" t="s">
         <v>37</v>
       </c>
-      <c r="E26">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="27" spans="2:7" x14ac:dyDescent="0.4">
-      <c r="C27" t="s">
+      <c r="E32" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="G32" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="33" spans="3:7" x14ac:dyDescent="0.4">
+      <c r="C33" t="s">
         <v>38</v>
       </c>
-      <c r="E27">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="28" spans="2:7" x14ac:dyDescent="0.4">
-      <c r="C28" t="s">
-        <v>39</v>
-      </c>
-      <c r="E28">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="29" spans="2:7" x14ac:dyDescent="0.4">
-      <c r="C29" t="s">
-        <v>40</v>
-      </c>
-      <c r="E29">
-        <v>360</v>
+      <c r="E33" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="G33" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="34" spans="3:7" x14ac:dyDescent="0.4">
+      <c r="C34" t="s">
+        <v>58</v>
+      </c>
+      <c r="E34" t="s">
+        <v>60</v>
+      </c>
+      <c r="G34" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="36" spans="3:7" x14ac:dyDescent="0.4">
+      <c r="G36" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="37" spans="3:7" x14ac:dyDescent="0.4">
+      <c r="G37" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="38" spans="3:7" x14ac:dyDescent="0.4">
+      <c r="G38" t="s">
+        <v>65</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto update: 2026-09-06 11:24:04
</commit_message>
<xml_diff>
--- a/docs/成績計算.xlsx
+++ b/docs/成績計算.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Dev\CDY_YAKYULIFE\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4F4A22E6-5399-4B53-A284-0B7080BC2447}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{04A45B3F-1AE6-49C0-8D18-D035DB8AA8AD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="4160" yWindow="380" windowWidth="28800" windowHeight="15910" xr2:uid="{AA24EB7E-E109-46F7-B027-D52B85957C16}"/>
   </bookViews>
@@ -117,18 +117,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>2B = min(AB, round(50 * (AB / 600.0) * min(1.05, ((con + spd * 2.0) - 3 * (par - 59)) / 225.0) * noise)) + round[-3, +3]</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>3B = min(AB, round(30 * (AB / 600.0) * min(1.05, ((pow + con + spd * 3.0) - 5 * (par - 59)) / 375.0) * noise)) + round[-3, +3]</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>HR = min(AB, round(80 * (AB / 600.0) * min(1.05, ((con + pow * 2.0) - 3 * (par - 59)) / 225.0) * noise)) + round[-3, +3]</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>R = round(140 * min(1.05, (HR * 1.00 + (3B * 0.70 + 2B * 0.45 + (H - 2B - 3B - HR) * 0.25 + BB * 0.20) * min(1.05, (spd - (par - 59)) / 75.0)) / 140.0) * noise) + round[-3, +3]</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -302,6 +290,18 @@
   </si>
   <si>
     <t>類似野手的守位降位，養成/二軍也比照野手</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>HR = min(H, round(80 * (AB / 600.0) * min(1.05, ((con + pow * 2.0) - 3 * (par - 59)) / 225.0) * noise)) + round[-3, +3]</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>3B = min(H - HR, round(30 * (AB / 600.0) * min(1.05, ((pow + con + spd * 3.0) - 5 * (par - 59)) / 375.0) * noise)) + round[-3, +3]</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>2B = min(H - 3B - 2B, round(50 * (AB / 600.0) * min(1.05, ((con + spd * 2.0) - 3 * (par - 59)) / 225.0) * noise)) + round[-3, +3]</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -708,7 +708,7 @@
   <sheetData>
     <row r="2" spans="2:12" x14ac:dyDescent="0.4">
       <c r="B2" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="C2" t="s">
         <v>0</v>
@@ -717,7 +717,7 @@
         <v>162</v>
       </c>
       <c r="H2" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
     </row>
     <row r="3" spans="2:12" x14ac:dyDescent="0.4">
@@ -759,7 +759,7 @@
         <v>140</v>
       </c>
       <c r="G5" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
     </row>
     <row r="6" spans="2:12" x14ac:dyDescent="0.4">
@@ -802,7 +802,7 @@
         <v>50</v>
       </c>
       <c r="G8" t="s">
-        <v>19</v>
+        <v>65</v>
       </c>
     </row>
     <row r="9" spans="2:12" x14ac:dyDescent="0.4">
@@ -816,7 +816,7 @@
         <v>30</v>
       </c>
       <c r="G9" t="s">
-        <v>20</v>
+        <v>64</v>
       </c>
     </row>
     <row r="10" spans="2:12" x14ac:dyDescent="0.4">
@@ -830,7 +830,7 @@
         <v>80</v>
       </c>
       <c r="G10" t="s">
-        <v>21</v>
+        <v>63</v>
       </c>
     </row>
     <row r="11" spans="2:12" x14ac:dyDescent="0.4">
@@ -858,7 +858,7 @@
         <v>120</v>
       </c>
       <c r="G12" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
     </row>
     <row r="13" spans="2:12" x14ac:dyDescent="0.4">
@@ -872,7 +872,7 @@
         <v>220</v>
       </c>
       <c r="G13" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
     </row>
     <row r="14" spans="2:12" x14ac:dyDescent="0.4">
@@ -886,7 +886,7 @@
         <v>80</v>
       </c>
       <c r="G14" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
     </row>
     <row r="15" spans="2:12" x14ac:dyDescent="0.4">
@@ -900,188 +900,188 @@
         <v>30</v>
       </c>
       <c r="G15" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
     </row>
     <row r="18" spans="2:8" x14ac:dyDescent="0.4">
       <c r="B18" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="C18" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="G18" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="H18" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
     </row>
     <row r="19" spans="2:8" x14ac:dyDescent="0.4">
       <c r="C19" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="G19" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="H19" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
     </row>
     <row r="20" spans="2:8" x14ac:dyDescent="0.4">
       <c r="C20" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="E20">
         <v>25</v>
       </c>
       <c r="G20" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
     </row>
     <row r="21" spans="2:8" x14ac:dyDescent="0.4">
       <c r="C21" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="E21">
         <v>20</v>
       </c>
       <c r="G21" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
     </row>
     <row r="22" spans="2:8" x14ac:dyDescent="0.4">
       <c r="C22" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="E22">
         <v>65</v>
       </c>
       <c r="G22" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
     </row>
     <row r="23" spans="2:8" x14ac:dyDescent="0.4">
       <c r="C23" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="E23">
         <v>40</v>
       </c>
       <c r="G23" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
     </row>
     <row r="24" spans="2:8" x14ac:dyDescent="0.4">
       <c r="C24" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="E24">
         <v>260</v>
       </c>
       <c r="G24" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
     </row>
     <row r="25" spans="2:8" x14ac:dyDescent="0.4">
       <c r="G25" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
     </row>
     <row r="26" spans="2:8" x14ac:dyDescent="0.4">
       <c r="G26" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
     </row>
     <row r="27" spans="2:8" x14ac:dyDescent="0.4">
       <c r="G27" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
     </row>
     <row r="28" spans="2:8" x14ac:dyDescent="0.4">
       <c r="G28" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
     </row>
     <row r="29" spans="2:8" x14ac:dyDescent="0.4">
       <c r="C29" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="E29">
         <v>260</v>
       </c>
       <c r="G29" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
     </row>
     <row r="30" spans="2:8" x14ac:dyDescent="0.4">
       <c r="C30" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="E30">
         <v>150</v>
       </c>
       <c r="G30" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
     </row>
     <row r="31" spans="2:8" x14ac:dyDescent="0.4">
       <c r="C31" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="E31">
         <v>140</v>
       </c>
       <c r="G31" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
     </row>
     <row r="32" spans="2:8" x14ac:dyDescent="0.4">
       <c r="C32" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="E32" s="2" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="G32" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
     </row>
     <row r="33" spans="3:7" x14ac:dyDescent="0.4">
       <c r="C33" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="E33" s="2" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="G33" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
     </row>
     <row r="34" spans="3:7" x14ac:dyDescent="0.4">
       <c r="C34" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="E34" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="G34" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
     </row>
     <row r="36" spans="3:7" x14ac:dyDescent="0.4">
       <c r="G36" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
     </row>
     <row r="37" spans="3:7" x14ac:dyDescent="0.4">
       <c r="G37" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
     </row>
     <row r="38" spans="3:7" x14ac:dyDescent="0.4">
       <c r="G38" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
     </row>
   </sheetData>

</xml_diff>